<commit_message>
revisi gabung data dan testing data baru 2026
</commit_message>
<xml_diff>
--- a/output/training_result_databaru/frequent_itemsets_60_40.xlsx
+++ b/output/training_result_databaru/frequent_itemsets_60_40.xlsx
@@ -1416,7 +1416,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>frozenset({'operator_Anisa', 'waktu_Siang'})</t>
+          <t>frozenset({'waktu_Siang', 'operator_Anisa'})</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>frozenset({'produk_hb night brightening', 'waktu_Siang'})</t>
+          <t>frozenset({'waktu_Siang', 'produk_hb night brightening'})</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>frozenset({'waktu_Siang', 'operator_Indah'})</t>
+          <t>frozenset({'operator_Indah', 'waktu_Siang'})</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>frozenset({'produk_paket brightening', 'waktu_Siang'})</t>
+          <t>frozenset({'waktu_Siang', 'produk_paket brightening'})</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>frozenset({'produk_paket brightening', 'operator_Indah'})</t>
+          <t>frozenset({'operator_Indah', 'produk_paket brightening'})</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>frozenset({'waktu_Pagi', 'produk_paket brightening'})</t>
+          <t>frozenset({'produk_paket brightening', 'waktu_Pagi'})</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>frozenset({'produk_sunscreen oily acne new', 'operator_Indah'})</t>
+          <t>frozenset({'operator_Indah', 'produk_sunscreen oily acne new'})</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -1722,7 +1722,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>frozenset({'waktu_Pagi', 'produk_sunscreen oily acne new'})</t>
+          <t>frozenset({'produk_sunscreen oily acne new', 'waktu_Pagi'})</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -1740,7 +1740,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>frozenset({'operator_Oktavira', 'produk_sunscreen oily acne new'})</t>
+          <t>frozenset({'produk_sunscreen oily acne new', 'operator_Oktavira'})</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>frozenset({'produk_sunscreen oily acne new', 'waktu_Siang', 'operator_Indah'})</t>
+          <t>frozenset({'operator_Indah', 'produk_sunscreen oily acne new', 'waktu_Siang'})</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>frozenset({'waktu_Malam', 'produk_sunscreen oily acne new', 'operator_Indah'})</t>
+          <t>frozenset({'operator_Indah', 'produk_sunscreen oily acne new', 'waktu_Malam'})</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>frozenset({'operator_Oktavira', 'waktu_Siang', 'produk_sunscreen oily acne new'})</t>
+          <t>frozenset({'produk_sunscreen oily acne new', 'operator_Oktavira', 'waktu_Siang'})</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -1812,7 +1812,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>frozenset({'waktu_Pagi', 'operator_Riska'})</t>
+          <t>frozenset({'operator_Riska', 'waktu_Pagi'})</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -1884,7 +1884,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>frozenset({'waktu_Malam', 'operator_Indah'})</t>
+          <t>frozenset({'operator_Indah', 'waktu_Malam'})</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -1902,7 +1902,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>frozenset({'waktu_Pagi', 'operator_Indah'})</t>
+          <t>frozenset({'operator_Indah', 'waktu_Pagi'})</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>frozenset({'waktu_Pagi', 'operator_Oktavira'})</t>
+          <t>frozenset({'operator_Oktavira', 'waktu_Pagi'})</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>frozenset({'produk_serum brightening glowing', 'operator_Riska'})</t>
+          <t>frozenset({'operator_Riska', 'produk_serum brightening glowing'})</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>frozenset({'produk_serum brightening glowing', 'waktu_Siang'})</t>
+          <t>frozenset({'waktu_Siang', 'produk_serum brightening glowing'})</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>frozenset({'produk_serum brightening glowing', 'operator_Oktavira'})</t>
+          <t>frozenset({'operator_Oktavira', 'produk_serum brightening glowing'})</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -2082,7 +2082,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>frozenset({'operator_Riska', 'produk_night cream brightening'})</t>
+          <t>frozenset({'produk_night cream brightening', 'operator_Riska'})</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2136,7 +2136,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>frozenset({'waktu_Pagi', 'produk_night cream brightening'})</t>
+          <t>frozenset({'produk_night cream brightening', 'waktu_Pagi'})</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -2172,7 +2172,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>frozenset({'waktu_Siang', 'operator_Riska', 'produk_night cream brightening'})</t>
+          <t>frozenset({'waktu_Siang', 'produk_night cream brightening', 'operator_Riska'})</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -2190,7 +2190,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>frozenset({'waktu_Siang', 'operator_Indah', 'produk_night cream brightening'})</t>
+          <t>frozenset({'operator_Indah', 'waktu_Siang', 'produk_night cream brightening'})</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -2208,7 +2208,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>frozenset({'waktu_Pagi', 'operator_Oktavira', 'produk_night cream brightening'})</t>
+          <t>frozenset({'operator_Oktavira', 'produk_night cream brightening', 'waktu_Pagi'})</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -2244,7 +2244,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>frozenset({'waktu_Pagi', 'produk_sunscreen glowing new'})</t>
+          <t>frozenset({'produk_sunscreen glowing new', 'waktu_Pagi'})</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -2280,7 +2280,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>frozenset({'produk_hb dosting 75 gram', 'waktu_Siang'})</t>
+          <t>frozenset({'waktu_Siang', 'produk_hb dosting 75 gram'})</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>frozenset({'produk_hb dosting 75 gram', 'operator_Indah'})</t>
+          <t>frozenset({'operator_Indah', 'produk_hb dosting 75 gram'})</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -2334,7 +2334,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>frozenset({'produk_hb dosting 75 gram', 'operator_Oktavira'})</t>
+          <t>frozenset({'operator_Oktavira', 'produk_hb dosting 75 gram'})</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>frozenset({'produk_daily ceramois hydra gel', 'waktu_Siang'})</t>
+          <t>frozenset({'waktu_Siang', 'produk_daily ceramois hydra gel'})</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -2370,7 +2370,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>frozenset({'produk_daily ceramois hydra gel', 'operator_Indah'})</t>
+          <t>frozenset({'operator_Indah', 'produk_daily ceramois hydra gel'})</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -2388,7 +2388,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>frozenset({'produk_daily ceramois hydra gel', 'operator_Oktavira'})</t>
+          <t>frozenset({'operator_Oktavira', 'produk_daily ceramois hydra gel'})</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -2406,7 +2406,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>frozenset({'produk_daily ceramois hydra gel', 'produk_night cream brightening'})</t>
+          <t>frozenset({'produk_night cream brightening', 'produk_daily ceramois hydra gel'})</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -2442,7 +2442,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>frozenset({'waktu_Pagi', 'produk_daily ceramois hydra gel'})</t>
+          <t>frozenset({'produk_daily ceramois hydra gel', 'waktu_Pagi'})</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -2478,7 +2478,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>frozenset({'waktu_Siang', 'produk_daily ceramois hydra gel', 'operator_Riska'})</t>
+          <t>frozenset({'produk_daily ceramois hydra gel', 'waktu_Siang', 'operator_Riska'})</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -2496,7 +2496,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>frozenset({'produk_night cream acne brightening', 'waktu_Siang'})</t>
+          <t>frozenset({'waktu_Siang', 'produk_night cream acne brightening'})</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>frozenset({'produk_night cream acne brightening', 'produk_night cream brightening'})</t>
+          <t>frozenset({'produk_night cream brightening', 'produk_night cream acne brightening'})</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -2532,7 +2532,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>frozenset({'waktu_Siang', 'produk_paket radian brightening ultimate'})</t>
+          <t>frozenset({'produk_paket radian brightening ultimate', 'waktu_Siang'})</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -2550,7 +2550,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>frozenset({'produk_paket radian brightening ultimate', 'operator_Indah'})</t>
+          <t>frozenset({'operator_Indah', 'produk_paket radian brightening ultimate'})</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>frozenset({'produk_radian brightening ultimate', 'operator_Indah'})</t>
+          <t>frozenset({'operator_Indah', 'produk_radian brightening ultimate'})</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -2676,7 +2676,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>frozenset({'produk_radian brightening ultimate', 'operator_Riska'})</t>
+          <t>frozenset({'operator_Riska', 'produk_radian brightening ultimate'})</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>frozenset({'produk_radian brightening ultimate', 'waktu_Siang'})</t>
+          <t>frozenset({'waktu_Siang', 'produk_radian brightening ultimate'})</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -2748,7 +2748,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>frozenset({'produk_radian brightening ultimate', 'waktu_Siang', 'operator_Indah'})</t>
+          <t>frozenset({'operator_Indah', 'waktu_Siang', 'produk_radian brightening ultimate'})</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -2766,7 +2766,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>frozenset({'operator_Oktavira', 'produk_radian brightening ultimate', 'waktu_Siang'})</t>
+          <t>frozenset({'operator_Oktavira', 'waktu_Siang', 'produk_radian brightening ultimate'})</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -2784,7 +2784,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>frozenset({'waktu_Pagi', 'produk_sunscreen natural glow for normal skin new'})</t>
+          <t>frozenset({'produk_sunscreen natural glow for normal skin new', 'waktu_Pagi'})</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -2856,7 +2856,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>frozenset({'waktu_Pagi', 'produk_facial wash oily acne 110 ml new'})</t>
+          <t>frozenset({'produk_facial wash oily acne 110 ml new', 'waktu_Pagi'})</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -2874,7 +2874,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>frozenset({'produk_facial wash oily acne 110 ml new', 'operator_Oktavira'})</t>
+          <t>frozenset({'operator_Oktavira', 'produk_facial wash oily acne 110 ml new'})</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -2892,7 +2892,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>frozenset({'produk_facial wash oily acne 110 ml new', 'waktu_Siang'})</t>
+          <t>frozenset({'waktu_Siang', 'produk_facial wash oily acne 110 ml new'})</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -2910,7 +2910,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>frozenset({'produk_facial wash oily acne 110 ml new', 'operator_Indah'})</t>
+          <t>frozenset({'operator_Indah', 'produk_facial wash oily acne 110 ml new'})</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>frozenset({'waktu_Pagi', 'produk_facial wash oily acne 110 ml new', 'operator_Riska'})</t>
+          <t>frozenset({'produk_facial wash oily acne 110 ml new', 'operator_Riska', 'waktu_Pagi'})</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -2946,7 +2946,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>frozenset({'produk_brightening cream 1 with licorice plus astaxanthin', 'waktu_Siang'})</t>
+          <t>frozenset({'waktu_Siang', 'produk_brightening cream 1 with licorice plus astaxanthin'})</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -2964,7 +2964,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>frozenset({'produk_serum for acne skin new', 'waktu_Siang'})</t>
+          <t>frozenset({'waktu_Siang', 'produk_serum for acne skin new'})</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -3018,7 +3018,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>frozenset({'produk_paket acne brightening', 'operator_Indah'})</t>
+          <t>frozenset({'operator_Indah', 'produk_paket acne brightening'})</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -3054,7 +3054,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>frozenset({'produk_acne cream 2 new', 'waktu_Siang'})</t>
+          <t>frozenset({'waktu_Siang', 'produk_acne cream 2 new'})</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -3090,7 +3090,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>frozenset({'produk_hb night yellow plus licorice', 'operator_Indah'})</t>
+          <t>frozenset({'operator_Indah', 'produk_hb night yellow plus licorice'})</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -3126,7 +3126,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>frozenset({'produk_glowtech spicule rejuvenation', 'waktu_Siang'})</t>
+          <t>frozenset({'waktu_Siang', 'produk_glowtech spicule rejuvenation'})</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">

</xml_diff>